<commit_message>
perf: code splitting and memoization for performance
</commit_message>
<xml_diff>
--- a/ระบบลางาน ออนไลน์ 2025.xlsx
+++ b/ระบบลางาน ออนไลน์ 2025.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11835" activeTab="5"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11835" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Setting" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1744" uniqueCount="883">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1745" uniqueCount="884">
   <si>
     <t>Setting (Folder)</t>
   </si>
@@ -2675,6 +2675,9 @@
   </si>
   <si>
     <t>Sunday</t>
+  </si>
+  <si>
+    <t>ID</t>
   </si>
 </sst>
 </file>
@@ -2684,7 +2687,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d/m/yyyy"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -2768,8 +2771,12 @@
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <name val="Prompt"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2780,6 +2787,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF745AF2"/>
         <bgColor rgb="FF745AF2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -2796,7 +2809,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -2883,6 +2896,20 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -3181,15 +3208,16 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:K83"/>
+  <dimension ref="A1:L83"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="2" max="2" width="32.42578125" customWidth="1"/>
     <col min="4" max="4" width="17.42578125" customWidth="1"/>
-    <col min="9" max="9" width="60.5703125" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" style="42" customWidth="1"/>
+    <col min="10" max="10" width="60.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:12">
       <c r="A1" s="6" t="s">
         <v>14</v>
       </c>
@@ -3202,46 +3230,50 @@
       <c r="D1" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="38" t="s">
+        <v>883</v>
+      </c>
+      <c r="F1" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="G1" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="H1" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="I1" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="J1" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="K1" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="K1" s="10" t="s">
+      <c r="L1" s="10" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:12">
       <c r="A2" s="11" t="s">
         <v>25</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
       <c r="D2" s="12"/>
-      <c r="E2" s="13"/>
+      <c r="E2" s="39"/>
       <c r="F2" s="13"/>
       <c r="G2" s="13"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="15"/>
-      <c r="J2" s="16"/>
-      <c r="K2" s="17" t="b">
+      <c r="H2" s="13"/>
+      <c r="I2" s="14"/>
+      <c r="J2" s="15"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="17" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:12">
       <c r="A3" s="11" t="s">
         <v>26</v>
       </c>
@@ -3254,27 +3286,28 @@
       <c r="D3" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="E3" s="40"/>
+      <c r="F3" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="F3" s="13" t="s">
+      <c r="G3" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="G3" s="13" t="s">
+      <c r="H3" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="H3" s="14">
+      <c r="I3" s="14">
         <v>45838</v>
       </c>
-      <c r="I3" s="15" t="s">
+      <c r="J3" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="J3" s="16"/>
-      <c r="K3" s="17" t="b">
+      <c r="K3" s="16"/>
+      <c r="L3" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:12">
       <c r="A4" s="11" t="s">
         <v>34</v>
       </c>
@@ -3287,29 +3320,32 @@
       <c r="D4" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" s="41">
+        <v>160</v>
+      </c>
+      <c r="F4" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="G4" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="G4" s="13" t="s">
+      <c r="H4" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="H4" s="14">
+      <c r="I4" s="14">
         <v>45837</v>
       </c>
-      <c r="I4" s="15" t="s">
+      <c r="J4" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="J4" s="16" t="s">
+      <c r="K4" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="K4" s="17" t="b">
+      <c r="L4" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:12">
       <c r="A5" s="20" t="s">
         <v>43</v>
       </c>
@@ -3322,27 +3358,30 @@
       <c r="D5" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="E5" s="20" t="s">
+      <c r="E5" s="40">
+        <v>272</v>
+      </c>
+      <c r="F5" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="F5" s="20" t="s">
+      <c r="G5" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="G5" s="20" t="s">
+      <c r="H5" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="H5" s="14">
+      <c r="I5" s="14">
         <v>45838</v>
       </c>
-      <c r="I5" s="15" t="s">
+      <c r="J5" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="J5" s="16"/>
-      <c r="K5" s="17" t="b">
+      <c r="K5" s="16"/>
+      <c r="L5" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:12">
       <c r="A6" s="20" t="s">
         <v>48</v>
       </c>
@@ -3355,27 +3394,30 @@
       <c r="D6" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="E6" s="20" t="s">
+      <c r="E6" s="41">
+        <v>288</v>
+      </c>
+      <c r="F6" s="20" t="s">
         <v>52</v>
       </c>
-      <c r="F6" s="20" t="s">
+      <c r="G6" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G6" s="20" t="s">
+      <c r="H6" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="H6" s="14">
+      <c r="I6" s="14">
         <v>45839</v>
       </c>
-      <c r="I6" s="15" t="s">
+      <c r="J6" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="J6" s="16"/>
-      <c r="K6" s="17" t="b">
+      <c r="K6" s="16"/>
+      <c r="L6" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:12">
       <c r="A7" s="20" t="s">
         <v>55</v>
       </c>
@@ -3388,27 +3430,30 @@
       <c r="D7" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="E7" s="20" t="s">
+      <c r="E7" s="41">
+        <v>92</v>
+      </c>
+      <c r="F7" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="F7" s="20" t="s">
+      <c r="G7" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="G7" s="20" t="s">
+      <c r="H7" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="H7" s="14">
+      <c r="I7" s="14">
         <v>45838</v>
       </c>
-      <c r="I7" s="15" t="s">
+      <c r="J7" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="J7" s="16"/>
-      <c r="K7" s="17" t="b">
+      <c r="K7" s="16"/>
+      <c r="L7" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:12">
       <c r="A8" s="20" t="s">
         <v>61</v>
       </c>
@@ -3421,27 +3466,30 @@
       <c r="D8" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="E8" s="20" t="s">
+      <c r="E8" s="40">
+        <v>158</v>
+      </c>
+      <c r="F8" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="F8" s="20" t="s">
+      <c r="G8" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="G8" s="20" t="s">
+      <c r="H8" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H8" s="14">
+      <c r="I8" s="14">
         <v>45841</v>
       </c>
-      <c r="I8" s="15" t="s">
+      <c r="J8" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="J8" s="16"/>
-      <c r="K8" s="17" t="b">
+      <c r="K8" s="16"/>
+      <c r="L8" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:12">
       <c r="A9" s="20" t="s">
         <v>67</v>
       </c>
@@ -3454,27 +3502,30 @@
       <c r="D9" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="E9" s="20" t="s">
+      <c r="E9" s="40">
+        <v>161</v>
+      </c>
+      <c r="F9" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="F9" s="20" t="s">
+      <c r="G9" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="G9" s="20" t="s">
+      <c r="H9" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H9" s="14">
+      <c r="I9" s="14">
         <v>45841</v>
       </c>
-      <c r="I9" s="15" t="s">
+      <c r="J9" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="J9" s="16"/>
-      <c r="K9" s="17" t="b">
+      <c r="K9" s="16"/>
+      <c r="L9" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:12">
       <c r="A10" s="20" t="s">
         <v>72</v>
       </c>
@@ -3487,27 +3538,30 @@
       <c r="D10" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="E10" s="20" t="s">
+      <c r="E10" s="40">
+        <v>168</v>
+      </c>
+      <c r="F10" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="F10" s="20" t="s">
+      <c r="G10" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="G10" s="20" t="s">
+      <c r="H10" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H10" s="14">
+      <c r="I10" s="14">
         <v>45841</v>
       </c>
-      <c r="I10" s="15" t="s">
+      <c r="J10" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="J10" s="16"/>
-      <c r="K10" s="17" t="b">
+      <c r="K10" s="16"/>
+      <c r="L10" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:12">
       <c r="A11" s="20" t="s">
         <v>77</v>
       </c>
@@ -3520,27 +3574,30 @@
       <c r="D11" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="E11" s="20" t="s">
+      <c r="E11" s="40">
+        <v>195</v>
+      </c>
+      <c r="F11" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="F11" s="20" t="s">
+      <c r="G11" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="G11" s="20" t="s">
+      <c r="H11" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H11" s="14">
+      <c r="I11" s="14">
         <v>45841</v>
       </c>
-      <c r="I11" s="15" t="s">
+      <c r="J11" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="J11" s="16"/>
-      <c r="K11" s="17" t="b">
+      <c r="K11" s="16"/>
+      <c r="L11" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:12">
       <c r="A12" s="20" t="s">
         <v>82</v>
       </c>
@@ -3553,27 +3610,30 @@
       <c r="D12" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="E12" s="20" t="s">
+      <c r="E12" s="40">
+        <v>198</v>
+      </c>
+      <c r="F12" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="F12" s="20" t="s">
+      <c r="G12" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="G12" s="20" t="s">
+      <c r="H12" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H12" s="14">
+      <c r="I12" s="14">
         <v>45841</v>
       </c>
-      <c r="I12" s="15" t="s">
+      <c r="J12" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="J12" s="16"/>
-      <c r="K12" s="17" t="b">
+      <c r="K12" s="16"/>
+      <c r="L12" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:12">
       <c r="A13" s="20" t="s">
         <v>87</v>
       </c>
@@ -3586,27 +3646,30 @@
       <c r="D13" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="E13" s="20" t="s">
+      <c r="E13" s="40">
+        <v>205</v>
+      </c>
+      <c r="F13" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="F13" s="20" t="s">
+      <c r="G13" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="G13" s="20" t="s">
+      <c r="H13" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H13" s="14">
+      <c r="I13" s="14">
         <v>45841</v>
       </c>
-      <c r="I13" s="15" t="s">
+      <c r="J13" s="15" t="s">
         <v>91</v>
       </c>
-      <c r="J13" s="16"/>
-      <c r="K13" s="17" t="b">
+      <c r="K13" s="16"/>
+      <c r="L13" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" spans="1:12">
       <c r="A14" s="20" t="s">
         <v>92</v>
       </c>
@@ -3619,27 +3682,30 @@
       <c r="D14" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="E14" s="20" t="s">
+      <c r="E14" s="40">
+        <v>217</v>
+      </c>
+      <c r="F14" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="F14" s="20" t="s">
+      <c r="G14" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="G14" s="20" t="s">
+      <c r="H14" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H14" s="14">
+      <c r="I14" s="14">
         <v>45841</v>
       </c>
-      <c r="I14" s="15" t="s">
+      <c r="J14" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="J14" s="16"/>
-      <c r="K14" s="17" t="b">
+      <c r="K14" s="16"/>
+      <c r="L14" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15" spans="1:12">
       <c r="A15" s="20" t="s">
         <v>97</v>
       </c>
@@ -3652,27 +3718,30 @@
       <c r="D15" s="18" t="s">
         <v>100</v>
       </c>
-      <c r="E15" s="20" t="s">
+      <c r="E15" s="40">
+        <v>224</v>
+      </c>
+      <c r="F15" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="F15" s="20" t="s">
+      <c r="G15" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="G15" s="20" t="s">
+      <c r="H15" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H15" s="14">
+      <c r="I15" s="14">
         <v>45841</v>
       </c>
-      <c r="I15" s="15" t="s">
+      <c r="J15" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="J15" s="16"/>
-      <c r="K15" s="17" t="b">
+      <c r="K15" s="16"/>
+      <c r="L15" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16" spans="1:12">
       <c r="A16" s="20" t="s">
         <v>102</v>
       </c>
@@ -3685,44 +3754,48 @@
       <c r="D16" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="E16" s="20" t="s">
+      <c r="E16" s="40">
+        <v>228</v>
+      </c>
+      <c r="F16" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="F16" s="20" t="s">
+      <c r="G16" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="G16" s="20" t="s">
+      <c r="H16" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H16" s="14">
+      <c r="I16" s="14">
         <v>45841</v>
       </c>
-      <c r="I16" s="15" t="s">
+      <c r="J16" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="J16" s="16"/>
-      <c r="K16" s="17" t="b">
+      <c r="K16" s="16"/>
+      <c r="L16" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:11">
+    <row r="17" spans="1:12">
       <c r="A17" s="20" t="s">
         <v>107</v>
       </c>
       <c r="B17" s="12"/>
       <c r="C17" s="12"/>
       <c r="D17" s="12"/>
-      <c r="E17" s="20"/>
+      <c r="E17" s="41"/>
       <c r="F17" s="20"/>
       <c r="G17" s="20"/>
-      <c r="H17" s="14"/>
-      <c r="I17" s="15"/>
-      <c r="J17" s="16"/>
-      <c r="K17" s="17" t="b">
+      <c r="H17" s="20"/>
+      <c r="I17" s="14"/>
+      <c r="J17" s="15"/>
+      <c r="K17" s="16"/>
+      <c r="L17" s="17" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:11">
+    <row r="18" spans="1:12">
       <c r="A18" s="20" t="s">
         <v>108</v>
       </c>
@@ -3735,27 +3808,30 @@
       <c r="D18" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="E18" s="20" t="s">
+      <c r="E18" s="40">
+        <v>234</v>
+      </c>
+      <c r="F18" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="F18" s="20" t="s">
+      <c r="G18" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="G18" s="20" t="s">
+      <c r="H18" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H18" s="14">
+      <c r="I18" s="14">
         <v>45841</v>
       </c>
-      <c r="I18" s="15" t="s">
+      <c r="J18" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="J18" s="16"/>
-      <c r="K18" s="17" t="b">
+      <c r="K18" s="16"/>
+      <c r="L18" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:11">
+    <row r="19" spans="1:12">
       <c r="A19" s="20" t="s">
         <v>113</v>
       </c>
@@ -3768,27 +3844,30 @@
       <c r="D19" s="18" t="s">
         <v>116</v>
       </c>
-      <c r="E19" s="20" t="s">
+      <c r="E19" s="40">
+        <v>236</v>
+      </c>
+      <c r="F19" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="F19" s="20" t="s">
+      <c r="G19" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="G19" s="20" t="s">
+      <c r="H19" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H19" s="14">
+      <c r="I19" s="14">
         <v>45841</v>
       </c>
-      <c r="I19" s="15" t="s">
+      <c r="J19" s="15" t="s">
         <v>117</v>
       </c>
-      <c r="J19" s="16"/>
-      <c r="K19" s="17" t="b">
+      <c r="K19" s="16"/>
+      <c r="L19" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:11">
+    <row r="20" spans="1:12">
       <c r="A20" s="20" t="s">
         <v>118</v>
       </c>
@@ -3801,27 +3880,30 @@
       <c r="D20" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="E20" s="20" t="s">
+      <c r="E20" s="40">
+        <v>238</v>
+      </c>
+      <c r="F20" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="F20" s="20" t="s">
+      <c r="G20" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="G20" s="20" t="s">
+      <c r="H20" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H20" s="14">
+      <c r="I20" s="14">
         <v>45841</v>
       </c>
-      <c r="I20" s="15" t="s">
+      <c r="J20" s="15" t="s">
         <v>122</v>
       </c>
-      <c r="J20" s="16"/>
-      <c r="K20" s="17" t="b">
+      <c r="K20" s="16"/>
+      <c r="L20" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:11">
+    <row r="21" spans="1:12">
       <c r="A21" s="20" t="s">
         <v>123</v>
       </c>
@@ -3834,27 +3916,30 @@
       <c r="D21" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="E21" s="20" t="s">
+      <c r="E21" s="40">
+        <v>248</v>
+      </c>
+      <c r="F21" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="F21" s="20" t="s">
+      <c r="G21" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="G21" s="20" t="s">
+      <c r="H21" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H21" s="14">
+      <c r="I21" s="14">
         <v>45841</v>
       </c>
-      <c r="I21" s="15" t="s">
+      <c r="J21" s="15" t="s">
         <v>127</v>
       </c>
-      <c r="J21" s="16"/>
-      <c r="K21" s="17" t="b">
+      <c r="K21" s="16"/>
+      <c r="L21" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:11">
+    <row r="22" spans="1:12">
       <c r="A22" s="20" t="s">
         <v>128</v>
       </c>
@@ -3867,27 +3952,30 @@
       <c r="D22" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="E22" s="20" t="s">
+      <c r="E22" s="40">
+        <v>251</v>
+      </c>
+      <c r="F22" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="F22" s="20" t="s">
+      <c r="G22" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="G22" s="20" t="s">
+      <c r="H22" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H22" s="14">
+      <c r="I22" s="14">
         <v>45841</v>
       </c>
-      <c r="I22" s="15" t="s">
+      <c r="J22" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="J22" s="16"/>
-      <c r="K22" s="17" t="b">
+      <c r="K22" s="16"/>
+      <c r="L22" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:11">
+    <row r="23" spans="1:12">
       <c r="A23" s="20" t="s">
         <v>133</v>
       </c>
@@ -3900,27 +3988,30 @@
       <c r="D23" s="18" t="s">
         <v>136</v>
       </c>
-      <c r="E23" s="20" t="s">
+      <c r="E23" s="40">
+        <v>254</v>
+      </c>
+      <c r="F23" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="F23" s="20" t="s">
+      <c r="G23" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="G23" s="20" t="s">
+      <c r="H23" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H23" s="14">
+      <c r="I23" s="14">
         <v>45841</v>
       </c>
-      <c r="I23" s="15" t="s">
+      <c r="J23" s="15" t="s">
         <v>137</v>
       </c>
-      <c r="J23" s="16"/>
-      <c r="K23" s="17" t="b">
+      <c r="K23" s="16"/>
+      <c r="L23" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:11">
+    <row r="24" spans="1:12">
       <c r="A24" s="20" t="s">
         <v>138</v>
       </c>
@@ -3933,44 +4024,48 @@
       <c r="D24" s="18" t="s">
         <v>141</v>
       </c>
-      <c r="E24" s="20" t="s">
+      <c r="E24" s="40">
+        <v>266</v>
+      </c>
+      <c r="F24" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="F24" s="20" t="s">
+      <c r="G24" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="G24" s="20" t="s">
+      <c r="H24" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H24" s="14">
+      <c r="I24" s="14">
         <v>45841</v>
       </c>
-      <c r="I24" s="15" t="s">
+      <c r="J24" s="15" t="s">
         <v>142</v>
       </c>
-      <c r="J24" s="16"/>
-      <c r="K24" s="17" t="b">
+      <c r="K24" s="16"/>
+      <c r="L24" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:11">
+    <row r="25" spans="1:12">
       <c r="A25" s="20" t="s">
         <v>143</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="12"/>
       <c r="D25" s="12"/>
-      <c r="E25" s="20"/>
+      <c r="E25" s="41"/>
       <c r="F25" s="20"/>
       <c r="G25" s="20"/>
-      <c r="H25" s="14"/>
-      <c r="I25" s="15"/>
-      <c r="J25" s="16"/>
-      <c r="K25" s="17" t="b">
+      <c r="H25" s="20"/>
+      <c r="I25" s="14"/>
+      <c r="J25" s="15"/>
+      <c r="K25" s="16"/>
+      <c r="L25" s="17" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:11">
+    <row r="26" spans="1:12">
       <c r="A26" s="20" t="s">
         <v>144</v>
       </c>
@@ -3983,27 +4078,30 @@
       <c r="D26" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="E26" s="20" t="s">
+      <c r="E26" s="40">
+        <v>276</v>
+      </c>
+      <c r="F26" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="F26" s="20" t="s">
+      <c r="G26" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="G26" s="20" t="s">
+      <c r="H26" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H26" s="14">
+      <c r="I26" s="14">
         <v>45841</v>
       </c>
-      <c r="I26" s="15" t="s">
+      <c r="J26" s="15" t="s">
         <v>148</v>
       </c>
-      <c r="J26" s="16"/>
-      <c r="K26" s="17" t="b">
+      <c r="K26" s="16"/>
+      <c r="L26" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:11">
+    <row r="27" spans="1:12">
       <c r="A27" s="20" t="s">
         <v>149</v>
       </c>
@@ -4016,27 +4114,30 @@
       <c r="D27" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="E27" s="20" t="s">
+      <c r="E27" s="40">
+        <v>277</v>
+      </c>
+      <c r="F27" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="F27" s="20" t="s">
+      <c r="G27" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="G27" s="20" t="s">
+      <c r="H27" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H27" s="14">
+      <c r="I27" s="14">
         <v>45841</v>
       </c>
-      <c r="I27" s="15" t="s">
+      <c r="J27" s="15" t="s">
         <v>153</v>
       </c>
-      <c r="J27" s="16"/>
-      <c r="K27" s="17" t="b">
+      <c r="K27" s="16"/>
+      <c r="L27" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:11">
+    <row r="28" spans="1:12">
       <c r="A28" s="20" t="s">
         <v>154</v>
       </c>
@@ -4049,27 +4150,30 @@
       <c r="D28" s="18" t="s">
         <v>157</v>
       </c>
-      <c r="E28" s="20" t="s">
+      <c r="E28" s="40">
+        <v>278</v>
+      </c>
+      <c r="F28" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="F28" s="20" t="s">
+      <c r="G28" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="G28" s="20" t="s">
+      <c r="H28" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H28" s="14">
+      <c r="I28" s="14">
         <v>45841</v>
       </c>
-      <c r="I28" s="15" t="s">
+      <c r="J28" s="15" t="s">
         <v>158</v>
       </c>
-      <c r="J28" s="16"/>
-      <c r="K28" s="17" t="b">
+      <c r="K28" s="16"/>
+      <c r="L28" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:11">
+    <row r="29" spans="1:12">
       <c r="A29" s="20" t="s">
         <v>159</v>
       </c>
@@ -4082,27 +4186,30 @@
       <c r="D29" s="18" t="s">
         <v>162</v>
       </c>
-      <c r="E29" s="20" t="s">
+      <c r="E29" s="40">
+        <v>280</v>
+      </c>
+      <c r="F29" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="F29" s="20" t="s">
+      <c r="G29" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="G29" s="20" t="s">
+      <c r="H29" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H29" s="14">
+      <c r="I29" s="14">
         <v>45841</v>
       </c>
-      <c r="I29" s="15" t="s">
+      <c r="J29" s="15" t="s">
         <v>163</v>
       </c>
-      <c r="J29" s="16"/>
-      <c r="K29" s="17" t="b">
+      <c r="K29" s="16"/>
+      <c r="L29" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:11">
+    <row r="30" spans="1:12">
       <c r="A30" s="20" t="s">
         <v>164</v>
       </c>
@@ -4115,27 +4222,30 @@
       <c r="D30" s="18" t="s">
         <v>167</v>
       </c>
-      <c r="E30" s="20" t="s">
+      <c r="E30" s="40">
+        <v>65</v>
+      </c>
+      <c r="F30" s="20" t="s">
         <v>168</v>
       </c>
-      <c r="F30" s="20" t="s">
+      <c r="G30" s="20" t="s">
         <v>169</v>
       </c>
-      <c r="G30" s="20" t="s">
+      <c r="H30" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H30" s="14">
+      <c r="I30" s="14">
         <v>45843</v>
       </c>
-      <c r="I30" s="15" t="s">
+      <c r="J30" s="15" t="s">
         <v>170</v>
       </c>
-      <c r="J30" s="16"/>
-      <c r="K30" s="17" t="b">
+      <c r="K30" s="16"/>
+      <c r="L30" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:11">
+    <row r="31" spans="1:12">
       <c r="A31" s="20" t="s">
         <v>171</v>
       </c>
@@ -4148,27 +4258,30 @@
       <c r="D31" s="18" t="s">
         <v>174</v>
       </c>
-      <c r="E31" s="20" t="s">
+      <c r="E31" s="40">
+        <v>71</v>
+      </c>
+      <c r="F31" s="20" t="s">
         <v>175</v>
       </c>
-      <c r="F31" s="20" t="s">
+      <c r="G31" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G31" s="20" t="s">
+      <c r="H31" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="H31" s="14">
+      <c r="I31" s="14">
         <v>45843</v>
       </c>
-      <c r="I31" s="15" t="s">
+      <c r="J31" s="15" t="s">
         <v>176</v>
       </c>
-      <c r="J31" s="16"/>
-      <c r="K31" s="17" t="b">
+      <c r="K31" s="16"/>
+      <c r="L31" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:11">
+    <row r="32" spans="1:12">
       <c r="A32" s="20" t="s">
         <v>177</v>
       </c>
@@ -4181,27 +4294,30 @@
       <c r="D32" s="18" t="s">
         <v>180</v>
       </c>
-      <c r="E32" s="20" t="s">
+      <c r="E32" s="40">
+        <v>76</v>
+      </c>
+      <c r="F32" s="20" t="s">
         <v>168</v>
       </c>
-      <c r="F32" s="20" t="s">
+      <c r="G32" s="20" t="s">
         <v>169</v>
       </c>
-      <c r="G32" s="20" t="s">
+      <c r="H32" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H32" s="14">
+      <c r="I32" s="14">
         <v>45843</v>
       </c>
-      <c r="I32" s="15" t="s">
+      <c r="J32" s="15" t="s">
         <v>181</v>
       </c>
-      <c r="J32" s="16"/>
-      <c r="K32" s="17" t="b">
+      <c r="K32" s="16"/>
+      <c r="L32" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:11">
+    <row r="33" spans="1:12">
       <c r="A33" s="20" t="s">
         <v>182</v>
       </c>
@@ -4214,27 +4330,28 @@
       <c r="D33" s="18" t="s">
         <v>185</v>
       </c>
-      <c r="E33" s="20" t="s">
+      <c r="E33" s="43"/>
+      <c r="F33" s="20" t="s">
         <v>168</v>
       </c>
-      <c r="F33" s="20" t="s">
+      <c r="G33" s="20" t="s">
         <v>169</v>
       </c>
-      <c r="G33" s="20" t="s">
+      <c r="H33" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H33" s="14">
+      <c r="I33" s="14">
         <v>45843</v>
       </c>
-      <c r="I33" s="15" t="s">
+      <c r="J33" s="15" t="s">
         <v>186</v>
       </c>
-      <c r="J33" s="16"/>
-      <c r="K33" s="17" t="b">
+      <c r="K33" s="16"/>
+      <c r="L33" s="17" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:11">
+    <row r="34" spans="1:12">
       <c r="A34" s="20" t="s">
         <v>187</v>
       </c>
@@ -4247,27 +4364,30 @@
       <c r="D34" s="18" t="s">
         <v>190</v>
       </c>
-      <c r="E34" s="20" t="s">
+      <c r="E34" s="40">
+        <v>77</v>
+      </c>
+      <c r="F34" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="F34" s="20" t="s">
+      <c r="G34" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="G34" s="20" t="s">
+      <c r="H34" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H34" s="14">
+      <c r="I34" s="14">
         <v>45843</v>
       </c>
-      <c r="I34" s="15" t="s">
+      <c r="J34" s="15" t="s">
         <v>191</v>
       </c>
-      <c r="J34" s="16"/>
-      <c r="K34" s="17" t="b">
+      <c r="K34" s="16"/>
+      <c r="L34" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:11">
+    <row r="35" spans="1:12">
       <c r="A35" s="20" t="s">
         <v>192</v>
       </c>
@@ -4280,27 +4400,30 @@
       <c r="D35" s="18" t="s">
         <v>195</v>
       </c>
-      <c r="E35" s="20" t="s">
+      <c r="E35" s="40">
+        <v>79</v>
+      </c>
+      <c r="F35" s="20" t="s">
         <v>196</v>
       </c>
-      <c r="F35" s="20" t="s">
+      <c r="G35" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G35" s="20" t="s">
+      <c r="H35" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H35" s="14">
+      <c r="I35" s="14">
         <v>45843</v>
       </c>
-      <c r="I35" s="15" t="s">
+      <c r="J35" s="15" t="s">
         <v>197</v>
       </c>
-      <c r="J35" s="16"/>
-      <c r="K35" s="17" t="b">
+      <c r="K35" s="16"/>
+      <c r="L35" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:11">
+    <row r="36" spans="1:12">
       <c r="A36" s="20" t="s">
         <v>198</v>
       </c>
@@ -4313,27 +4436,30 @@
       <c r="D36" s="18" t="s">
         <v>201</v>
       </c>
-      <c r="E36" s="20" t="s">
+      <c r="E36" s="40">
+        <v>101</v>
+      </c>
+      <c r="F36" s="20" t="s">
         <v>196</v>
       </c>
-      <c r="F36" s="20" t="s">
+      <c r="G36" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G36" s="20" t="s">
+      <c r="H36" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="H36" s="14">
+      <c r="I36" s="14">
         <v>45843</v>
       </c>
-      <c r="I36" s="15" t="s">
+      <c r="J36" s="15" t="s">
         <v>202</v>
       </c>
-      <c r="J36" s="16"/>
-      <c r="K36" s="17" t="b">
+      <c r="K36" s="16"/>
+      <c r="L36" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:11">
+    <row r="37" spans="1:12">
       <c r="A37" s="20" t="s">
         <v>203</v>
       </c>
@@ -4346,27 +4472,30 @@
       <c r="D37" s="18" t="s">
         <v>206</v>
       </c>
-      <c r="E37" s="20" t="s">
+      <c r="E37" s="40">
+        <v>106</v>
+      </c>
+      <c r="F37" s="20" t="s">
         <v>175</v>
       </c>
-      <c r="F37" s="20" t="s">
+      <c r="G37" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G37" s="20" t="s">
+      <c r="H37" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H37" s="14">
+      <c r="I37" s="14">
         <v>45843</v>
       </c>
-      <c r="I37" s="15" t="s">
+      <c r="J37" s="15" t="s">
         <v>207</v>
       </c>
-      <c r="J37" s="16"/>
-      <c r="K37" s="17" t="b">
+      <c r="K37" s="16"/>
+      <c r="L37" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:11">
+    <row r="38" spans="1:12">
       <c r="A38" s="20" t="s">
         <v>208</v>
       </c>
@@ -4379,27 +4508,30 @@
       <c r="D38" s="18" t="s">
         <v>211</v>
       </c>
-      <c r="E38" s="20" t="s">
+      <c r="E38" s="40">
+        <v>114</v>
+      </c>
+      <c r="F38" s="20" t="s">
         <v>168</v>
       </c>
-      <c r="F38" s="20" t="s">
+      <c r="G38" s="20" t="s">
         <v>169</v>
       </c>
-      <c r="G38" s="20" t="s">
+      <c r="H38" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H38" s="14">
+      <c r="I38" s="14">
         <v>45843</v>
       </c>
-      <c r="I38" s="15" t="s">
+      <c r="J38" s="15" t="s">
         <v>212</v>
       </c>
-      <c r="J38" s="16"/>
-      <c r="K38" s="17" t="b">
+      <c r="K38" s="16"/>
+      <c r="L38" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:11">
+    <row r="39" spans="1:12">
       <c r="A39" s="20" t="s">
         <v>213</v>
       </c>
@@ -4412,27 +4544,30 @@
       <c r="D39" s="18" t="s">
         <v>216</v>
       </c>
-      <c r="E39" s="20" t="s">
+      <c r="E39" s="40">
+        <v>122</v>
+      </c>
+      <c r="F39" s="20" t="s">
         <v>196</v>
       </c>
-      <c r="F39" s="20" t="s">
+      <c r="G39" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G39" s="20" t="s">
+      <c r="H39" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H39" s="14">
+      <c r="I39" s="14">
         <v>45843</v>
       </c>
-      <c r="I39" s="15" t="s">
+      <c r="J39" s="15" t="s">
         <v>217</v>
       </c>
-      <c r="J39" s="16"/>
-      <c r="K39" s="17" t="b">
+      <c r="K39" s="16"/>
+      <c r="L39" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:11">
+    <row r="40" spans="1:12">
       <c r="A40" s="20" t="s">
         <v>218</v>
       </c>
@@ -4445,27 +4580,30 @@
       <c r="D40" s="18" t="s">
         <v>221</v>
       </c>
-      <c r="E40" s="20" t="s">
+      <c r="E40" s="40">
+        <v>137</v>
+      </c>
+      <c r="F40" s="20" t="s">
         <v>196</v>
       </c>
-      <c r="F40" s="20" t="s">
+      <c r="G40" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G40" s="20" t="s">
+      <c r="H40" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H40" s="14">
+      <c r="I40" s="14">
         <v>45843</v>
       </c>
-      <c r="I40" s="15" t="s">
+      <c r="J40" s="15" t="s">
         <v>222</v>
       </c>
-      <c r="J40" s="16"/>
-      <c r="K40" s="17" t="b">
+      <c r="K40" s="16"/>
+      <c r="L40" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:11">
+    <row r="41" spans="1:12">
       <c r="A41" s="20" t="s">
         <v>223</v>
       </c>
@@ -4478,27 +4616,30 @@
       <c r="D41" s="18" t="s">
         <v>226</v>
       </c>
-      <c r="E41" s="20" t="s">
+      <c r="E41" s="40">
+        <v>141</v>
+      </c>
+      <c r="F41" s="20" t="s">
         <v>196</v>
       </c>
-      <c r="F41" s="20" t="s">
+      <c r="G41" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G41" s="20" t="s">
+      <c r="H41" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H41" s="14">
+      <c r="I41" s="14">
         <v>45843</v>
       </c>
-      <c r="I41" s="15" t="s">
+      <c r="J41" s="15" t="s">
         <v>227</v>
       </c>
-      <c r="J41" s="16"/>
-      <c r="K41" s="17" t="b">
+      <c r="K41" s="16"/>
+      <c r="L41" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:11">
+    <row r="42" spans="1:12">
       <c r="A42" s="20" t="s">
         <v>228</v>
       </c>
@@ -4511,27 +4652,30 @@
       <c r="D42" s="18" t="s">
         <v>231</v>
       </c>
-      <c r="E42" s="20" t="s">
+      <c r="E42" s="40">
+        <v>147</v>
+      </c>
+      <c r="F42" s="20" t="s">
         <v>175</v>
       </c>
-      <c r="F42" s="20" t="s">
+      <c r="G42" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G42" s="20" t="s">
+      <c r="H42" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H42" s="14">
+      <c r="I42" s="14">
         <v>45843</v>
       </c>
-      <c r="I42" s="15" t="s">
+      <c r="J42" s="15" t="s">
         <v>232</v>
       </c>
-      <c r="J42" s="16"/>
-      <c r="K42" s="17" t="b">
+      <c r="K42" s="16"/>
+      <c r="L42" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:11">
+    <row r="43" spans="1:12">
       <c r="A43" s="20" t="s">
         <v>233</v>
       </c>
@@ -4544,27 +4688,30 @@
       <c r="D43" s="18" t="s">
         <v>236</v>
       </c>
-      <c r="E43" s="20" t="s">
+      <c r="E43" s="40">
+        <v>153</v>
+      </c>
+      <c r="F43" s="20" t="s">
         <v>175</v>
       </c>
-      <c r="F43" s="20" t="s">
+      <c r="G43" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G43" s="20" t="s">
+      <c r="H43" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H43" s="14">
+      <c r="I43" s="14">
         <v>45843</v>
       </c>
-      <c r="I43" s="15" t="s">
+      <c r="J43" s="15" t="s">
         <v>237</v>
       </c>
-      <c r="J43" s="16"/>
-      <c r="K43" s="17" t="b">
+      <c r="K43" s="16"/>
+      <c r="L43" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:11">
+    <row r="44" spans="1:12">
       <c r="A44" s="20" t="s">
         <v>238</v>
       </c>
@@ -4577,27 +4724,30 @@
       <c r="D44" s="18" t="s">
         <v>241</v>
       </c>
-      <c r="E44" s="20" t="s">
+      <c r="E44" s="40">
+        <v>167</v>
+      </c>
+      <c r="F44" s="20" t="s">
         <v>196</v>
       </c>
-      <c r="F44" s="20" t="s">
+      <c r="G44" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G44" s="20" t="s">
+      <c r="H44" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H44" s="14">
+      <c r="I44" s="14">
         <v>45843</v>
       </c>
-      <c r="I44" s="15" t="s">
+      <c r="J44" s="15" t="s">
         <v>242</v>
       </c>
-      <c r="J44" s="16"/>
-      <c r="K44" s="17" t="b">
+      <c r="K44" s="16"/>
+      <c r="L44" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:11">
+    <row r="45" spans="1:12">
       <c r="A45" s="20" t="s">
         <v>243</v>
       </c>
@@ -4610,27 +4760,30 @@
       <c r="D45" s="18" t="s">
         <v>246</v>
       </c>
-      <c r="E45" s="20" t="s">
+      <c r="E45" s="40">
+        <v>169</v>
+      </c>
+      <c r="F45" s="20" t="s">
         <v>247</v>
       </c>
-      <c r="F45" s="20" t="s">
+      <c r="G45" s="20" t="s">
         <v>248</v>
       </c>
-      <c r="G45" s="20" t="s">
+      <c r="H45" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="H45" s="14">
+      <c r="I45" s="14">
         <v>45843</v>
       </c>
-      <c r="I45" s="15" t="s">
+      <c r="J45" s="15" t="s">
         <v>249</v>
       </c>
-      <c r="J45" s="16"/>
-      <c r="K45" s="17" t="b">
+      <c r="K45" s="16"/>
+      <c r="L45" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:11">
+    <row r="46" spans="1:12">
       <c r="A46" s="20" t="s">
         <v>250</v>
       </c>
@@ -4643,27 +4796,30 @@
       <c r="D46" s="18" t="s">
         <v>253</v>
       </c>
-      <c r="E46" s="20" t="s">
+      <c r="E46" s="40">
+        <v>187</v>
+      </c>
+      <c r="F46" s="20" t="s">
         <v>254</v>
       </c>
-      <c r="F46" s="20" t="s">
+      <c r="G46" s="20" t="s">
         <v>169</v>
       </c>
-      <c r="G46" s="20" t="s">
+      <c r="H46" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="H46" s="14">
+      <c r="I46" s="14">
         <v>45843</v>
       </c>
-      <c r="I46" s="15" t="s">
+      <c r="J46" s="15" t="s">
         <v>255</v>
       </c>
-      <c r="J46" s="16"/>
-      <c r="K46" s="17" t="b">
+      <c r="K46" s="16"/>
+      <c r="L46" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:11">
+    <row r="47" spans="1:12">
       <c r="A47" s="20" t="s">
         <v>256</v>
       </c>
@@ -4676,27 +4832,30 @@
       <c r="D47" s="18" t="s">
         <v>259</v>
       </c>
-      <c r="E47" s="20" t="s">
+      <c r="E47" s="40">
+        <v>192</v>
+      </c>
+      <c r="F47" s="20" t="s">
         <v>168</v>
       </c>
-      <c r="F47" s="20" t="s">
+      <c r="G47" s="20" t="s">
         <v>169</v>
       </c>
-      <c r="G47" s="20" t="s">
+      <c r="H47" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H47" s="14">
+      <c r="I47" s="14">
         <v>45843</v>
       </c>
-      <c r="I47" s="15" t="s">
+      <c r="J47" s="15" t="s">
         <v>260</v>
       </c>
-      <c r="J47" s="16"/>
-      <c r="K47" s="17" t="b">
+      <c r="K47" s="16"/>
+      <c r="L47" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:11">
+    <row r="48" spans="1:12">
       <c r="A48" s="20" t="s">
         <v>261</v>
       </c>
@@ -4709,27 +4868,30 @@
       <c r="D48" s="18" t="s">
         <v>264</v>
       </c>
-      <c r="E48" s="20" t="s">
+      <c r="E48" s="40">
+        <v>193</v>
+      </c>
+      <c r="F48" s="20" t="s">
         <v>196</v>
       </c>
-      <c r="F48" s="20" t="s">
+      <c r="G48" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G48" s="20" t="s">
+      <c r="H48" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H48" s="14">
+      <c r="I48" s="14">
         <v>45843</v>
       </c>
-      <c r="I48" s="15" t="s">
+      <c r="J48" s="15" t="s">
         <v>265</v>
       </c>
-      <c r="J48" s="16"/>
-      <c r="K48" s="17" t="b">
+      <c r="K48" s="16"/>
+      <c r="L48" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:11">
+    <row r="49" spans="1:12">
       <c r="A49" s="20" t="s">
         <v>266</v>
       </c>
@@ -4742,27 +4904,30 @@
       <c r="D49" s="18" t="s">
         <v>269</v>
       </c>
-      <c r="E49" s="20" t="s">
+      <c r="E49" s="40">
+        <v>196</v>
+      </c>
+      <c r="F49" s="20" t="s">
         <v>175</v>
       </c>
-      <c r="F49" s="20" t="s">
+      <c r="G49" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G49" s="20" t="s">
+      <c r="H49" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H49" s="14">
+      <c r="I49" s="14">
         <v>45843</v>
       </c>
-      <c r="I49" s="15" t="s">
+      <c r="J49" s="15" t="s">
         <v>270</v>
       </c>
-      <c r="J49" s="16"/>
-      <c r="K49" s="17" t="b">
+      <c r="K49" s="16"/>
+      <c r="L49" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:11">
+    <row r="50" spans="1:12">
       <c r="A50" s="20" t="s">
         <v>271</v>
       </c>
@@ -4775,27 +4940,30 @@
       <c r="D50" s="18" t="s">
         <v>274</v>
       </c>
-      <c r="E50" s="20" t="s">
+      <c r="E50" s="40">
+        <v>197</v>
+      </c>
+      <c r="F50" s="20" t="s">
         <v>168</v>
       </c>
-      <c r="F50" s="20" t="s">
+      <c r="G50" s="20" t="s">
         <v>169</v>
       </c>
-      <c r="G50" s="20" t="s">
+      <c r="H50" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H50" s="14">
+      <c r="I50" s="14">
         <v>45843</v>
       </c>
-      <c r="I50" s="15" t="s">
+      <c r="J50" s="15" t="s">
         <v>275</v>
       </c>
-      <c r="J50" s="16"/>
-      <c r="K50" s="17" t="b">
+      <c r="K50" s="16"/>
+      <c r="L50" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:11">
+    <row r="51" spans="1:12">
       <c r="A51" s="20" t="s">
         <v>276</v>
       </c>
@@ -4808,27 +4976,30 @@
       <c r="D51" s="18" t="s">
         <v>279</v>
       </c>
-      <c r="E51" s="20" t="s">
+      <c r="E51" s="40">
+        <v>203</v>
+      </c>
+      <c r="F51" s="20" t="s">
         <v>175</v>
       </c>
-      <c r="F51" s="20" t="s">
+      <c r="G51" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G51" s="20" t="s">
+      <c r="H51" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H51" s="14">
+      <c r="I51" s="14">
         <v>45843</v>
       </c>
-      <c r="I51" s="15" t="s">
+      <c r="J51" s="15" t="s">
         <v>280</v>
       </c>
-      <c r="J51" s="16"/>
-      <c r="K51" s="17" t="b">
+      <c r="K51" s="16"/>
+      <c r="L51" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:11">
+    <row r="52" spans="1:12">
       <c r="A52" s="20" t="s">
         <v>281</v>
       </c>
@@ -4841,27 +5012,30 @@
       <c r="D52" s="18" t="s">
         <v>284</v>
       </c>
-      <c r="E52" s="20" t="s">
+      <c r="E52" s="40">
+        <v>206</v>
+      </c>
+      <c r="F52" s="20" t="s">
         <v>196</v>
       </c>
-      <c r="F52" s="20" t="s">
+      <c r="G52" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G52" s="20" t="s">
+      <c r="H52" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H52" s="14">
+      <c r="I52" s="14">
         <v>45843</v>
       </c>
-      <c r="I52" s="15" t="s">
+      <c r="J52" s="15" t="s">
         <v>285</v>
       </c>
-      <c r="J52" s="16"/>
-      <c r="K52" s="17" t="b">
+      <c r="K52" s="16"/>
+      <c r="L52" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:11">
+    <row r="53" spans="1:12">
       <c r="A53" s="20" t="s">
         <v>286</v>
       </c>
@@ -4874,27 +5048,30 @@
       <c r="D53" s="18" t="s">
         <v>289</v>
       </c>
-      <c r="E53" s="20" t="s">
+      <c r="E53" s="40">
+        <v>213</v>
+      </c>
+      <c r="F53" s="20" t="s">
         <v>196</v>
       </c>
-      <c r="F53" s="20" t="s">
+      <c r="G53" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G53" s="20" t="s">
+      <c r="H53" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H53" s="14">
+      <c r="I53" s="14">
         <v>45843</v>
       </c>
-      <c r="I53" s="15" t="s">
+      <c r="J53" s="15" t="s">
         <v>290</v>
       </c>
-      <c r="J53" s="16"/>
-      <c r="K53" s="17" t="b">
+      <c r="K53" s="16"/>
+      <c r="L53" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:11">
+    <row r="54" spans="1:12">
       <c r="A54" s="20" t="s">
         <v>291</v>
       </c>
@@ -4907,27 +5084,30 @@
       <c r="D54" s="18" t="s">
         <v>294</v>
       </c>
-      <c r="E54" s="20" t="s">
+      <c r="E54" s="40">
+        <v>214</v>
+      </c>
+      <c r="F54" s="20" t="s">
         <v>295</v>
       </c>
-      <c r="F54" s="20" t="s">
+      <c r="G54" s="20" t="s">
         <v>296</v>
       </c>
-      <c r="G54" s="20" t="s">
+      <c r="H54" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="H54" s="14">
+      <c r="I54" s="14">
         <v>45843</v>
       </c>
-      <c r="I54" s="15" t="s">
+      <c r="J54" s="15" t="s">
         <v>297</v>
       </c>
-      <c r="J54" s="16"/>
-      <c r="K54" s="17" t="b">
+      <c r="K54" s="16"/>
+      <c r="L54" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:11">
+    <row r="55" spans="1:12">
       <c r="A55" s="20" t="s">
         <v>298</v>
       </c>
@@ -4940,27 +5120,30 @@
       <c r="D55" s="18" t="s">
         <v>301</v>
       </c>
-      <c r="E55" s="20" t="s">
+      <c r="E55" s="40">
+        <v>223</v>
+      </c>
+      <c r="F55" s="20" t="s">
         <v>196</v>
       </c>
-      <c r="F55" s="20" t="s">
+      <c r="G55" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G55" s="20" t="s">
+      <c r="H55" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H55" s="14">
+      <c r="I55" s="14">
         <v>45843</v>
       </c>
-      <c r="I55" s="15" t="s">
+      <c r="J55" s="15" t="s">
         <v>302</v>
       </c>
-      <c r="J55" s="16"/>
-      <c r="K55" s="17" t="b">
+      <c r="K55" s="16"/>
+      <c r="L55" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:11">
+    <row r="56" spans="1:12">
       <c r="A56" s="20" t="s">
         <v>303</v>
       </c>
@@ -4973,27 +5156,30 @@
       <c r="D56" s="18" t="s">
         <v>306</v>
       </c>
-      <c r="E56" s="20" t="s">
+      <c r="E56" s="40">
+        <v>235</v>
+      </c>
+      <c r="F56" s="20" t="s">
         <v>196</v>
       </c>
-      <c r="F56" s="20" t="s">
+      <c r="G56" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G56" s="20" t="s">
+      <c r="H56" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H56" s="14">
+      <c r="I56" s="14">
         <v>45843</v>
       </c>
-      <c r="I56" s="15" t="s">
+      <c r="J56" s="15" t="s">
         <v>307</v>
       </c>
-      <c r="J56" s="16"/>
-      <c r="K56" s="17" t="b">
+      <c r="K56" s="16"/>
+      <c r="L56" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:11">
+    <row r="57" spans="1:12">
       <c r="A57" s="20" t="s">
         <v>308</v>
       </c>
@@ -5006,27 +5192,30 @@
       <c r="D57" s="18" t="s">
         <v>311</v>
       </c>
-      <c r="E57" s="20" t="s">
+      <c r="E57" s="40">
+        <v>240</v>
+      </c>
+      <c r="F57" s="20" t="s">
         <v>196</v>
       </c>
-      <c r="F57" s="20" t="s">
+      <c r="G57" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G57" s="20" t="s">
+      <c r="H57" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H57" s="14">
+      <c r="I57" s="14">
         <v>45843</v>
       </c>
-      <c r="I57" s="15" t="s">
+      <c r="J57" s="15" t="s">
         <v>312</v>
       </c>
-      <c r="J57" s="16"/>
-      <c r="K57" s="17" t="b">
+      <c r="K57" s="16"/>
+      <c r="L57" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:11">
+    <row r="58" spans="1:12">
       <c r="A58" s="20" t="s">
         <v>313</v>
       </c>
@@ -5039,27 +5228,30 @@
       <c r="D58" s="18" t="s">
         <v>316</v>
       </c>
-      <c r="E58" s="20" t="s">
+      <c r="E58" s="40">
+        <v>242</v>
+      </c>
+      <c r="F58" s="20" t="s">
         <v>196</v>
       </c>
-      <c r="F58" s="20" t="s">
+      <c r="G58" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G58" s="20" t="s">
+      <c r="H58" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H58" s="14">
+      <c r="I58" s="14">
         <v>45843</v>
       </c>
-      <c r="I58" s="15" t="s">
+      <c r="J58" s="15" t="s">
         <v>317</v>
       </c>
-      <c r="J58" s="16"/>
-      <c r="K58" s="17" t="b">
+      <c r="K58" s="16"/>
+      <c r="L58" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:11">
+    <row r="59" spans="1:12">
       <c r="A59" s="20" t="s">
         <v>318</v>
       </c>
@@ -5072,27 +5264,30 @@
       <c r="D59" s="18" t="s">
         <v>321</v>
       </c>
-      <c r="E59" s="20" t="s">
+      <c r="E59" s="40">
+        <v>246</v>
+      </c>
+      <c r="F59" s="20" t="s">
         <v>168</v>
       </c>
-      <c r="F59" s="20" t="s">
+      <c r="G59" s="20" t="s">
         <v>169</v>
       </c>
-      <c r="G59" s="20" t="s">
+      <c r="H59" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H59" s="14">
+      <c r="I59" s="14">
         <v>45843</v>
       </c>
-      <c r="I59" s="15" t="s">
+      <c r="J59" s="15" t="s">
         <v>322</v>
       </c>
-      <c r="J59" s="16"/>
-      <c r="K59" s="17" t="b">
+      <c r="K59" s="16"/>
+      <c r="L59" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:11">
+    <row r="60" spans="1:12">
       <c r="A60" s="20" t="s">
         <v>323</v>
       </c>
@@ -5105,27 +5300,28 @@
       <c r="D60" s="18" t="s">
         <v>326</v>
       </c>
-      <c r="E60" s="20" t="s">
+      <c r="E60" s="40"/>
+      <c r="F60" s="20" t="s">
         <v>175</v>
       </c>
-      <c r="F60" s="20" t="s">
+      <c r="G60" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G60" s="20" t="s">
+      <c r="H60" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H60" s="14">
+      <c r="I60" s="14">
         <v>45843</v>
       </c>
-      <c r="I60" s="15" t="s">
+      <c r="J60" s="15" t="s">
         <v>327</v>
       </c>
-      <c r="J60" s="16"/>
-      <c r="K60" s="17" t="b">
+      <c r="K60" s="16"/>
+      <c r="L60" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:11">
+    <row r="61" spans="1:12">
       <c r="A61" s="20" t="s">
         <v>328</v>
       </c>
@@ -5138,27 +5334,30 @@
       <c r="D61" s="18" t="s">
         <v>331</v>
       </c>
-      <c r="E61" s="20" t="s">
+      <c r="E61" s="40">
+        <v>261</v>
+      </c>
+      <c r="F61" s="20" t="s">
         <v>175</v>
       </c>
-      <c r="F61" s="20" t="s">
+      <c r="G61" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G61" s="20" t="s">
+      <c r="H61" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H61" s="14">
+      <c r="I61" s="14">
         <v>45843</v>
       </c>
-      <c r="I61" s="15" t="s">
+      <c r="J61" s="15" t="s">
         <v>332</v>
       </c>
-      <c r="J61" s="16"/>
-      <c r="K61" s="17" t="b">
+      <c r="K61" s="16"/>
+      <c r="L61" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:11">
+    <row r="62" spans="1:12">
       <c r="A62" s="20" t="s">
         <v>333</v>
       </c>
@@ -5171,27 +5370,30 @@
       <c r="D62" s="18" t="s">
         <v>336</v>
       </c>
-      <c r="E62" s="20" t="s">
+      <c r="E62" s="40">
+        <v>262</v>
+      </c>
+      <c r="F62" s="20" t="s">
         <v>175</v>
       </c>
-      <c r="F62" s="20" t="s">
+      <c r="G62" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G62" s="20" t="s">
+      <c r="H62" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H62" s="14">
+      <c r="I62" s="14">
         <v>45843</v>
       </c>
-      <c r="I62" s="15" t="s">
+      <c r="J62" s="15" t="s">
         <v>337</v>
       </c>
-      <c r="J62" s="16"/>
-      <c r="K62" s="17" t="b">
+      <c r="K62" s="16"/>
+      <c r="L62" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:11">
+    <row r="63" spans="1:12">
       <c r="A63" s="20" t="s">
         <v>338</v>
       </c>
@@ -5204,27 +5406,30 @@
       <c r="D63" s="18" t="s">
         <v>341</v>
       </c>
-      <c r="E63" s="20" t="s">
+      <c r="E63" s="40">
+        <v>264</v>
+      </c>
+      <c r="F63" s="20" t="s">
         <v>196</v>
       </c>
-      <c r="F63" s="20" t="s">
+      <c r="G63" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G63" s="20" t="s">
+      <c r="H63" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H63" s="14">
+      <c r="I63" s="14">
         <v>45843</v>
       </c>
-      <c r="I63" s="15" t="s">
+      <c r="J63" s="15" t="s">
         <v>342</v>
       </c>
-      <c r="J63" s="16"/>
-      <c r="K63" s="17" t="b">
+      <c r="K63" s="16"/>
+      <c r="L63" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:11">
+    <row r="64" spans="1:12">
       <c r="A64" s="20" t="s">
         <v>343</v>
       </c>
@@ -5237,27 +5442,30 @@
       <c r="D64" s="18" t="s">
         <v>346</v>
       </c>
-      <c r="E64" s="20" t="s">
+      <c r="E64" s="40">
+        <v>265</v>
+      </c>
+      <c r="F64" s="20" t="s">
         <v>168</v>
       </c>
-      <c r="F64" s="20" t="s">
+      <c r="G64" s="20" t="s">
         <v>169</v>
       </c>
-      <c r="G64" s="20" t="s">
+      <c r="H64" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H64" s="14">
+      <c r="I64" s="14">
         <v>45843</v>
       </c>
-      <c r="I64" s="15" t="s">
+      <c r="J64" s="15" t="s">
         <v>347</v>
       </c>
-      <c r="J64" s="16"/>
-      <c r="K64" s="17" t="b">
+      <c r="K64" s="16"/>
+      <c r="L64" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:11">
+    <row r="65" spans="1:12">
       <c r="A65" s="20" t="s">
         <v>348</v>
       </c>
@@ -5270,44 +5478,48 @@
       <c r="D65" s="18" t="s">
         <v>351</v>
       </c>
-      <c r="E65" s="20" t="s">
+      <c r="E65" s="40">
+        <v>270</v>
+      </c>
+      <c r="F65" s="20" t="s">
         <v>196</v>
       </c>
-      <c r="F65" s="20" t="s">
+      <c r="G65" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G65" s="20" t="s">
+      <c r="H65" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H65" s="14">
+      <c r="I65" s="14">
         <v>45843</v>
       </c>
-      <c r="I65" s="15" t="s">
+      <c r="J65" s="15" t="s">
         <v>352</v>
       </c>
-      <c r="J65" s="16"/>
-      <c r="K65" s="17" t="b">
+      <c r="K65" s="16"/>
+      <c r="L65" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:11">
+    <row r="66" spans="1:12">
       <c r="A66" s="20" t="s">
         <v>353</v>
       </c>
       <c r="B66" s="12"/>
       <c r="C66" s="12"/>
       <c r="D66" s="12"/>
-      <c r="E66" s="20"/>
+      <c r="E66" s="41"/>
       <c r="F66" s="20"/>
       <c r="G66" s="20"/>
-      <c r="H66" s="14"/>
-      <c r="I66" s="15"/>
-      <c r="J66" s="16"/>
-      <c r="K66" s="17" t="b">
+      <c r="H66" s="20"/>
+      <c r="I66" s="14"/>
+      <c r="J66" s="15"/>
+      <c r="K66" s="16"/>
+      <c r="L66" s="17" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:11">
+    <row r="67" spans="1:12">
       <c r="A67" s="20" t="s">
         <v>354</v>
       </c>
@@ -5320,27 +5532,30 @@
       <c r="D67" s="12" t="s">
         <v>357</v>
       </c>
-      <c r="E67" s="20" t="s">
+      <c r="E67" s="41">
+        <v>281</v>
+      </c>
+      <c r="F67" s="20" t="s">
         <v>196</v>
       </c>
-      <c r="F67" s="20" t="s">
+      <c r="G67" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G67" s="20" t="s">
+      <c r="H67" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H67" s="14">
+      <c r="I67" s="14">
         <v>45843</v>
       </c>
-      <c r="I67" s="15" t="s">
+      <c r="J67" s="15" t="s">
         <v>358</v>
       </c>
-      <c r="J67" s="16"/>
-      <c r="K67" s="17" t="b">
+      <c r="K67" s="16"/>
+      <c r="L67" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:11">
+    <row r="68" spans="1:12">
       <c r="A68" s="20" t="s">
         <v>359</v>
       </c>
@@ -5353,27 +5568,30 @@
       <c r="D68" s="18" t="s">
         <v>362</v>
       </c>
-      <c r="E68" s="20" t="s">
+      <c r="E68" s="40">
+        <v>284</v>
+      </c>
+      <c r="F68" s="20" t="s">
         <v>175</v>
       </c>
-      <c r="F68" s="20" t="s">
+      <c r="G68" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G68" s="20" t="s">
+      <c r="H68" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H68" s="14">
+      <c r="I68" s="14">
         <v>45843</v>
       </c>
-      <c r="I68" s="15" t="s">
+      <c r="J68" s="15" t="s">
         <v>363</v>
       </c>
-      <c r="J68" s="16"/>
-      <c r="K68" s="17" t="b">
+      <c r="K68" s="16"/>
+      <c r="L68" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:11">
+    <row r="69" spans="1:12">
       <c r="A69" s="20" t="s">
         <v>364</v>
       </c>
@@ -5386,27 +5604,30 @@
       <c r="D69" s="18" t="s">
         <v>367</v>
       </c>
-      <c r="E69" s="20" t="s">
+      <c r="E69" s="40">
+        <v>285</v>
+      </c>
+      <c r="F69" s="20" t="s">
         <v>168</v>
       </c>
-      <c r="F69" s="20" t="s">
+      <c r="G69" s="20" t="s">
         <v>169</v>
       </c>
-      <c r="G69" s="20" t="s">
+      <c r="H69" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H69" s="14">
+      <c r="I69" s="14">
         <v>45843</v>
       </c>
-      <c r="I69" s="15" t="s">
+      <c r="J69" s="15" t="s">
         <v>368</v>
       </c>
-      <c r="J69" s="16"/>
-      <c r="K69" s="17" t="b">
+      <c r="K69" s="16"/>
+      <c r="L69" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:11">
+    <row r="70" spans="1:12">
       <c r="A70" s="20" t="s">
         <v>369</v>
       </c>
@@ -5419,27 +5640,30 @@
       <c r="D70" s="18" t="s">
         <v>372</v>
       </c>
-      <c r="E70" s="20" t="s">
+      <c r="E70" s="40">
+        <v>286</v>
+      </c>
+      <c r="F70" s="20" t="s">
         <v>196</v>
       </c>
-      <c r="F70" s="20" t="s">
+      <c r="G70" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G70" s="20" t="s">
+      <c r="H70" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H70" s="14">
+      <c r="I70" s="14">
         <v>45843</v>
       </c>
-      <c r="I70" s="15" t="s">
+      <c r="J70" s="15" t="s">
         <v>373</v>
       </c>
-      <c r="J70" s="16"/>
-      <c r="K70" s="17" t="b">
+      <c r="K70" s="16"/>
+      <c r="L70" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:11">
+    <row r="71" spans="1:12">
       <c r="A71" s="20" t="s">
         <v>374</v>
       </c>
@@ -5452,27 +5676,28 @@
       <c r="D71" s="18" t="s">
         <v>377</v>
       </c>
-      <c r="E71" s="20" t="s">
+      <c r="E71" s="40"/>
+      <c r="F71" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="F71" s="20" t="s">
+      <c r="G71" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="G71" s="20" t="s">
+      <c r="H71" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="H71" s="14">
+      <c r="I71" s="14">
         <v>45853</v>
       </c>
-      <c r="I71" s="15" t="s">
+      <c r="J71" s="15" t="s">
         <v>378</v>
       </c>
-      <c r="J71" s="16"/>
-      <c r="K71" s="17" t="b">
+      <c r="K71" s="16"/>
+      <c r="L71" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:11">
+    <row r="72" spans="1:12">
       <c r="A72" s="20" t="s">
         <v>379</v>
       </c>
@@ -5485,27 +5710,30 @@
       <c r="D72" s="18" t="s">
         <v>382</v>
       </c>
-      <c r="E72" s="20" t="s">
+      <c r="E72" s="40">
+        <v>289</v>
+      </c>
+      <c r="F72" s="20" t="s">
         <v>168</v>
       </c>
-      <c r="F72" s="20" t="s">
+      <c r="G72" s="20" t="s">
         <v>169</v>
       </c>
-      <c r="G72" s="20" t="s">
+      <c r="H72" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H72" s="14">
+      <c r="I72" s="14">
         <v>45871</v>
       </c>
-      <c r="I72" s="15" t="s">
+      <c r="J72" s="15" t="s">
         <v>383</v>
       </c>
-      <c r="J72" s="16"/>
-      <c r="K72" s="17" t="b">
+      <c r="K72" s="16"/>
+      <c r="L72" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:11">
+    <row r="73" spans="1:12">
       <c r="A73" s="20" t="s">
         <v>384</v>
       </c>
@@ -5518,27 +5746,30 @@
       <c r="D73" s="18" t="s">
         <v>387</v>
       </c>
-      <c r="E73" s="20" t="s">
+      <c r="E73" s="40">
+        <v>290</v>
+      </c>
+      <c r="F73" s="20" t="s">
         <v>196</v>
       </c>
-      <c r="F73" s="20" t="s">
+      <c r="G73" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G73" s="20" t="s">
+      <c r="H73" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H73" s="14">
+      <c r="I73" s="14">
         <v>45874</v>
       </c>
-      <c r="I73" s="15" t="s">
+      <c r="J73" s="15" t="s">
         <v>388</v>
       </c>
-      <c r="J73" s="16"/>
-      <c r="K73" s="17" t="b">
+      <c r="K73" s="16"/>
+      <c r="L73" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:11">
+    <row r="74" spans="1:12">
       <c r="A74" s="20" t="s">
         <v>389</v>
       </c>
@@ -5551,27 +5782,30 @@
       <c r="D74" s="18" t="s">
         <v>392</v>
       </c>
-      <c r="E74" s="20" t="s">
+      <c r="E74" s="40">
+        <v>291</v>
+      </c>
+      <c r="F74" s="20" t="s">
         <v>175</v>
       </c>
-      <c r="F74" s="20" t="s">
+      <c r="G74" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G74" s="20" t="s">
+      <c r="H74" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H74" s="14">
+      <c r="I74" s="14">
         <v>45904</v>
       </c>
-      <c r="I74" s="15" t="s">
+      <c r="J74" s="15" t="s">
         <v>393</v>
       </c>
-      <c r="J74" s="16"/>
-      <c r="K74" s="17" t="b">
+      <c r="K74" s="16"/>
+      <c r="L74" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:11">
+    <row r="75" spans="1:12">
       <c r="A75" s="20" t="s">
         <v>394</v>
       </c>
@@ -5584,27 +5818,30 @@
       <c r="D75" s="18" t="s">
         <v>397</v>
       </c>
-      <c r="E75" s="20" t="s">
+      <c r="E75" s="40">
+        <v>297</v>
+      </c>
+      <c r="F75" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="F75" s="20" t="s">
+      <c r="G75" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="G75" s="20" t="s">
+      <c r="H75" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H75" s="14">
+      <c r="I75" s="14">
         <v>46073</v>
       </c>
-      <c r="I75" s="15" t="s">
+      <c r="J75" s="15" t="s">
         <v>398</v>
       </c>
-      <c r="J75" s="16"/>
-      <c r="K75" s="17" t="b">
+      <c r="K75" s="16"/>
+      <c r="L75" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:11">
+    <row r="76" spans="1:12">
       <c r="A76" s="20" t="s">
         <v>399</v>
       </c>
@@ -5617,44 +5854,48 @@
       <c r="D76" s="18" t="s">
         <v>402</v>
       </c>
-      <c r="E76" s="20" t="s">
+      <c r="E76" s="40">
+        <v>261003</v>
+      </c>
+      <c r="F76" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="F76" s="20" t="s">
+      <c r="G76" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="G76" s="20" t="s">
+      <c r="H76" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H76" s="14">
+      <c r="I76" s="14">
         <v>46083</v>
       </c>
-      <c r="I76" s="15" t="s">
+      <c r="J76" s="15" t="s">
         <v>403</v>
       </c>
-      <c r="J76" s="16"/>
-      <c r="K76" s="17" t="b">
+      <c r="K76" s="16"/>
+      <c r="L76" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:11">
+    <row r="77" spans="1:12">
       <c r="A77" s="20" t="s">
         <v>404</v>
       </c>
       <c r="B77" s="12"/>
       <c r="C77" s="12"/>
       <c r="D77" s="12"/>
-      <c r="E77" s="20"/>
+      <c r="E77" s="41"/>
       <c r="F77" s="20"/>
       <c r="G77" s="20"/>
-      <c r="H77" s="14"/>
-      <c r="I77" s="15"/>
-      <c r="J77" s="16"/>
-      <c r="K77" s="17" t="b">
+      <c r="H77" s="20"/>
+      <c r="I77" s="14"/>
+      <c r="J77" s="15"/>
+      <c r="K77" s="16"/>
+      <c r="L77" s="17" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:11">
+    <row r="78" spans="1:12">
       <c r="A78" s="20" t="s">
         <v>405</v>
       </c>
@@ -5667,27 +5908,30 @@
       <c r="D78" s="18" t="s">
         <v>408</v>
       </c>
-      <c r="E78" s="20" t="s">
+      <c r="E78" s="40">
+        <v>292</v>
+      </c>
+      <c r="F78" s="20" t="s">
         <v>196</v>
       </c>
-      <c r="F78" s="20" t="s">
+      <c r="G78" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G78" s="20" t="s">
+      <c r="H78" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H78" s="14">
+      <c r="I78" s="14">
         <v>46115</v>
       </c>
-      <c r="I78" s="15" t="s">
+      <c r="J78" s="15" t="s">
         <v>409</v>
       </c>
-      <c r="J78" s="16"/>
-      <c r="K78" s="17" t="b">
+      <c r="K78" s="16"/>
+      <c r="L78" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:11">
+    <row r="79" spans="1:12">
       <c r="A79" s="20" t="s">
         <v>410</v>
       </c>
@@ -5700,27 +5944,30 @@
       <c r="D79" s="18" t="s">
         <v>413</v>
       </c>
-      <c r="E79" s="20" t="s">
+      <c r="E79" s="40">
+        <v>293</v>
+      </c>
+      <c r="F79" s="20" t="s">
         <v>168</v>
       </c>
-      <c r="F79" s="20" t="s">
+      <c r="G79" s="20" t="s">
         <v>169</v>
       </c>
-      <c r="G79" s="20" t="s">
+      <c r="H79" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="H79" s="14">
+      <c r="I79" s="14">
         <v>46140</v>
       </c>
-      <c r="I79" s="15" t="s">
+      <c r="J79" s="15" t="s">
         <v>414</v>
       </c>
-      <c r="J79" s="16"/>
-      <c r="K79" s="17" t="b">
+      <c r="K79" s="16"/>
+      <c r="L79" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:11">
+    <row r="80" spans="1:12">
       <c r="A80" s="20" t="s">
         <v>415</v>
       </c>
@@ -5733,27 +5980,28 @@
       <c r="D80" s="18" t="s">
         <v>418</v>
       </c>
-      <c r="E80" s="20" t="s">
+      <c r="E80" s="40"/>
+      <c r="F80" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="F80" s="20" t="s">
+      <c r="G80" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="G80" s="20" t="s">
+      <c r="H80" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H80" s="14">
+      <c r="I80" s="14">
         <v>46148</v>
       </c>
-      <c r="I80" s="15" t="s">
+      <c r="J80" s="15" t="s">
         <v>419</v>
       </c>
-      <c r="J80" s="16"/>
-      <c r="K80" s="17" t="b">
+      <c r="K80" s="16"/>
+      <c r="L80" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:11">
+    <row r="81" spans="1:12">
       <c r="A81" s="20" t="s">
         <v>420</v>
       </c>
@@ -5766,27 +6014,30 @@
       <c r="D81" s="18" t="s">
         <v>423</v>
       </c>
-      <c r="E81" s="20" t="s">
+      <c r="E81" s="40">
+        <v>295</v>
+      </c>
+      <c r="F81" s="20" t="s">
         <v>175</v>
       </c>
-      <c r="F81" s="20" t="s">
+      <c r="G81" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G81" s="20" t="s">
+      <c r="H81" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H81" s="14">
+      <c r="I81" s="14">
         <v>46179</v>
       </c>
-      <c r="I81" s="15" t="s">
+      <c r="J81" s="15" t="s">
         <v>424</v>
       </c>
-      <c r="J81" s="16"/>
-      <c r="K81" s="17" t="b">
+      <c r="K81" s="16"/>
+      <c r="L81" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:11">
+    <row r="82" spans="1:12">
       <c r="A82" s="20" t="s">
         <v>425</v>
       </c>
@@ -5799,27 +6050,30 @@
       <c r="D82" s="18" t="s">
         <v>428</v>
       </c>
-      <c r="E82" s="20" t="s">
+      <c r="E82" s="40">
+        <v>296</v>
+      </c>
+      <c r="F82" s="20" t="s">
         <v>175</v>
       </c>
-      <c r="F82" s="20" t="s">
+      <c r="G82" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="G82" s="20" t="s">
+      <c r="H82" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H82" s="14">
+      <c r="I82" s="14">
         <v>46192</v>
       </c>
-      <c r="I82" s="15" t="s">
+      <c r="J82" s="15" t="s">
         <v>429</v>
       </c>
-      <c r="J82" s="16"/>
-      <c r="K82" s="17" t="b">
+      <c r="K82" s="16"/>
+      <c r="L82" s="17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:11">
+    <row r="83" spans="1:12">
       <c r="A83" s="20" t="s">
         <v>430</v>
       </c>
@@ -5832,106 +6086,109 @@
       <c r="D83" s="18" t="s">
         <v>433</v>
       </c>
-      <c r="E83" s="20" t="s">
+      <c r="E83" s="40">
+        <v>298</v>
+      </c>
+      <c r="F83" s="20" t="s">
         <v>168</v>
       </c>
-      <c r="F83" s="20" t="s">
+      <c r="G83" s="20" t="s">
         <v>169</v>
       </c>
-      <c r="G83" s="20" t="s">
+      <c r="H83" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="H83" s="14">
+      <c r="I83" s="14">
         <v>46192</v>
       </c>
-      <c r="I83" s="15" t="s">
+      <c r="J83" s="15" t="s">
         <v>434</v>
       </c>
-      <c r="J83" s="16"/>
-      <c r="K83" s="17" t="b">
+      <c r="K83" s="16"/>
+      <c r="L83" s="17" t="b">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="I3" r:id="rId1"/>
-    <hyperlink ref="I4" r:id="rId2"/>
-    <hyperlink ref="J4" r:id="rId3"/>
-    <hyperlink ref="I5" r:id="rId4"/>
-    <hyperlink ref="I6" r:id="rId5"/>
-    <hyperlink ref="I7" r:id="rId6"/>
-    <hyperlink ref="I8" r:id="rId7"/>
-    <hyperlink ref="I9" r:id="rId8"/>
-    <hyperlink ref="I10" r:id="rId9"/>
-    <hyperlink ref="I11" r:id="rId10"/>
-    <hyperlink ref="I12" r:id="rId11"/>
-    <hyperlink ref="I13" r:id="rId12"/>
-    <hyperlink ref="I14" r:id="rId13"/>
-    <hyperlink ref="I15" r:id="rId14"/>
-    <hyperlink ref="I16" r:id="rId15"/>
-    <hyperlink ref="I18" r:id="rId16"/>
-    <hyperlink ref="I19" r:id="rId17"/>
-    <hyperlink ref="I20" r:id="rId18"/>
-    <hyperlink ref="I21" r:id="rId19"/>
-    <hyperlink ref="I22" r:id="rId20"/>
-    <hyperlink ref="I23" r:id="rId21"/>
-    <hyperlink ref="I24" r:id="rId22"/>
-    <hyperlink ref="I26" r:id="rId23"/>
-    <hyperlink ref="I27" r:id="rId24"/>
-    <hyperlink ref="I28" r:id="rId25"/>
-    <hyperlink ref="I29" r:id="rId26"/>
-    <hyperlink ref="I30" r:id="rId27"/>
-    <hyperlink ref="I31" r:id="rId28"/>
-    <hyperlink ref="I32" r:id="rId29"/>
-    <hyperlink ref="I33" r:id="rId30"/>
-    <hyperlink ref="I34" r:id="rId31"/>
-    <hyperlink ref="I35" r:id="rId32"/>
-    <hyperlink ref="I36" r:id="rId33"/>
-    <hyperlink ref="I37" r:id="rId34"/>
-    <hyperlink ref="I38" r:id="rId35"/>
-    <hyperlink ref="I39" r:id="rId36"/>
-    <hyperlink ref="I40" r:id="rId37"/>
-    <hyperlink ref="I41" r:id="rId38"/>
-    <hyperlink ref="I42" r:id="rId39"/>
-    <hyperlink ref="I43" r:id="rId40"/>
-    <hyperlink ref="I44" r:id="rId41"/>
-    <hyperlink ref="I45" r:id="rId42"/>
-    <hyperlink ref="I46" r:id="rId43"/>
-    <hyperlink ref="I47" r:id="rId44"/>
-    <hyperlink ref="I48" r:id="rId45"/>
-    <hyperlink ref="I49" r:id="rId46"/>
-    <hyperlink ref="I50" r:id="rId47"/>
-    <hyperlink ref="I51" r:id="rId48"/>
-    <hyperlink ref="I52" r:id="rId49"/>
-    <hyperlink ref="I53" r:id="rId50"/>
-    <hyperlink ref="I54" r:id="rId51"/>
-    <hyperlink ref="I55" r:id="rId52"/>
-    <hyperlink ref="I56" r:id="rId53"/>
-    <hyperlink ref="I57" r:id="rId54"/>
-    <hyperlink ref="I58" r:id="rId55"/>
-    <hyperlink ref="I59" r:id="rId56"/>
-    <hyperlink ref="I60" r:id="rId57"/>
-    <hyperlink ref="I61" r:id="rId58"/>
-    <hyperlink ref="I62" r:id="rId59"/>
-    <hyperlink ref="I63" r:id="rId60"/>
-    <hyperlink ref="I64" r:id="rId61"/>
-    <hyperlink ref="I65" r:id="rId62"/>
-    <hyperlink ref="I67" r:id="rId63"/>
-    <hyperlink ref="I68" r:id="rId64"/>
-    <hyperlink ref="I69" r:id="rId65"/>
-    <hyperlink ref="I70" r:id="rId66"/>
-    <hyperlink ref="I71" r:id="rId67"/>
-    <hyperlink ref="I72" r:id="rId68"/>
-    <hyperlink ref="I73" r:id="rId69"/>
-    <hyperlink ref="I74" r:id="rId70"/>
-    <hyperlink ref="I75" r:id="rId71"/>
-    <hyperlink ref="I76" r:id="rId72"/>
-    <hyperlink ref="I78" r:id="rId73"/>
-    <hyperlink ref="I79" r:id="rId74"/>
-    <hyperlink ref="I80" r:id="rId75"/>
-    <hyperlink ref="I81" r:id="rId76"/>
-    <hyperlink ref="I82" r:id="rId77"/>
-    <hyperlink ref="I83" r:id="rId78"/>
+    <hyperlink ref="J3" r:id="rId1"/>
+    <hyperlink ref="J4" r:id="rId2"/>
+    <hyperlink ref="K4" r:id="rId3"/>
+    <hyperlink ref="J5" r:id="rId4"/>
+    <hyperlink ref="J6" r:id="rId5"/>
+    <hyperlink ref="J7" r:id="rId6"/>
+    <hyperlink ref="J8" r:id="rId7"/>
+    <hyperlink ref="J9" r:id="rId8"/>
+    <hyperlink ref="J10" r:id="rId9"/>
+    <hyperlink ref="J11" r:id="rId10"/>
+    <hyperlink ref="J12" r:id="rId11"/>
+    <hyperlink ref="J13" r:id="rId12"/>
+    <hyperlink ref="J14" r:id="rId13"/>
+    <hyperlink ref="J15" r:id="rId14"/>
+    <hyperlink ref="J16" r:id="rId15"/>
+    <hyperlink ref="J18" r:id="rId16"/>
+    <hyperlink ref="J19" r:id="rId17"/>
+    <hyperlink ref="J20" r:id="rId18"/>
+    <hyperlink ref="J21" r:id="rId19"/>
+    <hyperlink ref="J22" r:id="rId20"/>
+    <hyperlink ref="J23" r:id="rId21"/>
+    <hyperlink ref="J24" r:id="rId22"/>
+    <hyperlink ref="J26" r:id="rId23"/>
+    <hyperlink ref="J27" r:id="rId24"/>
+    <hyperlink ref="J28" r:id="rId25"/>
+    <hyperlink ref="J29" r:id="rId26"/>
+    <hyperlink ref="J30" r:id="rId27"/>
+    <hyperlink ref="J31" r:id="rId28"/>
+    <hyperlink ref="J32" r:id="rId29"/>
+    <hyperlink ref="J33" r:id="rId30"/>
+    <hyperlink ref="J34" r:id="rId31"/>
+    <hyperlink ref="J35" r:id="rId32"/>
+    <hyperlink ref="J36" r:id="rId33"/>
+    <hyperlink ref="J37" r:id="rId34"/>
+    <hyperlink ref="J38" r:id="rId35"/>
+    <hyperlink ref="J39" r:id="rId36"/>
+    <hyperlink ref="J40" r:id="rId37"/>
+    <hyperlink ref="J41" r:id="rId38"/>
+    <hyperlink ref="J42" r:id="rId39"/>
+    <hyperlink ref="J43" r:id="rId40"/>
+    <hyperlink ref="J44" r:id="rId41"/>
+    <hyperlink ref="J45" r:id="rId42"/>
+    <hyperlink ref="J46" r:id="rId43"/>
+    <hyperlink ref="J47" r:id="rId44"/>
+    <hyperlink ref="J48" r:id="rId45"/>
+    <hyperlink ref="J49" r:id="rId46"/>
+    <hyperlink ref="J50" r:id="rId47"/>
+    <hyperlink ref="J51" r:id="rId48"/>
+    <hyperlink ref="J52" r:id="rId49"/>
+    <hyperlink ref="J53" r:id="rId50"/>
+    <hyperlink ref="J54" r:id="rId51"/>
+    <hyperlink ref="J55" r:id="rId52"/>
+    <hyperlink ref="J56" r:id="rId53"/>
+    <hyperlink ref="J57" r:id="rId54"/>
+    <hyperlink ref="J58" r:id="rId55"/>
+    <hyperlink ref="J59" r:id="rId56"/>
+    <hyperlink ref="J60" r:id="rId57"/>
+    <hyperlink ref="J61" r:id="rId58"/>
+    <hyperlink ref="J62" r:id="rId59"/>
+    <hyperlink ref="J63" r:id="rId60"/>
+    <hyperlink ref="J64" r:id="rId61"/>
+    <hyperlink ref="J65" r:id="rId62"/>
+    <hyperlink ref="J67" r:id="rId63"/>
+    <hyperlink ref="J68" r:id="rId64"/>
+    <hyperlink ref="J69" r:id="rId65"/>
+    <hyperlink ref="J70" r:id="rId66"/>
+    <hyperlink ref="J71" r:id="rId67"/>
+    <hyperlink ref="J72" r:id="rId68"/>
+    <hyperlink ref="J73" r:id="rId69"/>
+    <hyperlink ref="J74" r:id="rId70"/>
+    <hyperlink ref="J75" r:id="rId71"/>
+    <hyperlink ref="J76" r:id="rId72"/>
+    <hyperlink ref="J78" r:id="rId73"/>
+    <hyperlink ref="J79" r:id="rId74"/>
+    <hyperlink ref="J80" r:id="rId75"/>
+    <hyperlink ref="J81" r:id="rId76"/>
+    <hyperlink ref="J82" r:id="rId77"/>
+    <hyperlink ref="J83" r:id="rId78"/>
     <hyperlink ref="B7" r:id="rId79"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>